<commit_message>
docs(item10): marca CONCLUIDO fase 1 na fila — commit df4c998
Estado mudado citando o hash, conforme a propria regra 4 da fila: concluido
exige prova. FASE 1 apenas — a fase 2 (parar de aceitar o rotulo antigo) e
decisao do CEO e nao esta feita.

Conferidor limpo: 48 itens, nenhuma divergencia de estado.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DirXb1LNBwGEu4P2Gjbasv
</commit_message>
<xml_diff>
--- a/docs/LINHA_DE_PRODUCAO/PADAXOR_LINHA_DE_PRODUCAO_26.07.29.xlsx
+++ b/docs/LINHA_DE_PRODUCAO/PADAXOR_LINHA_DE_PRODUCAO_26.07.29.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">GLOSSARIO!$A$4:$E$38</definedName>
-    <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">HISTORICO!$A$4:$H$25</definedName>
+    <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">HISTORICO!$A$4:$H$26</definedName>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'LINHA DE PRODUCAO'!$A$4:$J$52</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="963" uniqueCount="635">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="971" uniqueCount="640">
   <si>
     <t xml:space="preserve">PADAXOR — Linha de Producao</t>
   </si>
@@ -228,264 +228,267 @@
     <t xml:space="preserve">scrypt-col$ e scrypt-pac$, com recusa ruidosa do prefixo errado.</t>
   </si>
   <si>
+    <t xml:space="preserve">fase 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FASE 1 entregue 30/07 no commit df4c998, 18 conferencias passando. Grava scrypt-col$ e scrypt-pac$, LE o scrypt$ antigo com a derivacao historica de cada esquema — ninguem trancado fora. Rotulo do outro esquema tem recusa ruidosa. FASE 2 (parar de aceitar scrypt$) e decisao do CEO, so quando nao houver mais hash antigo. NAO PUBLICADO: aguarda validacao.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Existem dois tipos de senha no sistema, guardados de jeitos diferentes, mas gravados com a MESMA etiqueta. E como dois frascos de remedio com o mesmo rotulo e conteudo diferente. Foi isso que fez seu login falhar por uma noite inteira. Isso poe rotulo diferente em cada frasco.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tela de login dentro do padaxor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tela propria chamando /api/collaborator/login e setCollabSession. O encanamento ja existe em collab-auth.ts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entregue 30/07 no commit 3a38349, conferido: pages/login/index.tsx criado e CollaboratorGate passou a redirecionar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tela de entrada propria do sistema, em vez da caixinha cinza do navegador. Ja entregue em 30/07.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site vira botao, nao segundo login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O login do site aponta para a tela do sistema em vez de autenticar por conta propria.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIBERADO em 30/07: a tela do item 11 existe. Elimina o segundo formulario de autenticacao.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O botao Entrar do site deixa de pedir senha por conta propria e passa a levar a pessoa para a tela de entrada do sistema. Uma porta so em vez de duas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DNS do padaxor.com.br no Cloudflare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trocar os servidores de nome no Registro.br pelos do Cloudflare.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Railway exige CNAME Flattening ou ALIAS para dominio raiz. Registro.br nao faz.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trocar quem cuida do endereco padaxor.com.br na internet. O registrador brasileiro nao faz um recurso que o servidor precisa; o Cloudflare faz, e e de graca.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dominio proprio apontando para o sistema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">app.padaxor.com.br no Railway com certificado automatico.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AGUARDANDO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Depende do passo do Cloudflare.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fazer app.padaxor.com.br apontar para o sistema, com cadeado de seguranca automatico no navegador.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marca PAXTER para PADAXOR no painel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O painel do sistema ainda exibe PAXTER na identidade visual.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">parcial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Titulo da aba e do aplicativo entregues 30/07 no commit 3a38349. As telas internas seguem no item 38.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O painel ainda mostrava o nome antigo PAXTER. Titulo da aba corrigido em 30/07; o resto das telas segue no item 38.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Porta da area do paciente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O site nao tem entrada para /api/area-paciente, que tem 12 rotas prontas no servidor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quarta porta do produto inteira sem macaneta.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O servidor ja tem doze portas prontas para a area do paciente, mas o site nao tem nenhum botao que leve ate elas. E uma porta inteira construida e sem macaneta.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indice unico em lower(login_username)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Impede dois colaboradores com o mesmo usuario. Erro 23505 traduzido em 409.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prevencao. Nao foi a causa do bug de hoje — nao havia duplicata.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Impedir que dois colaboradores tenham o mesmo nome de usuario. Prevencao: nao foi a causa do problema de hoje, mas seria a causa do de amanha.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ligar o registro de consumo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comecar a gravar em consumo_eventos, que ja existe com empresa_id, custo e idempotencia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P2 medio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sem historico nao ha painel. Historico nao se cria retroativamente. Espera o RLS do Dr. Code.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comecar a anotar quanto cada clinica usa do sistema. Sem anotar desde ja, nao existe historico depois: historico nao se cria para tras.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Catalogo de modulos com precos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tabela de modulos: nome, beneficio, valor de adesao, valor promocional, mensalidade.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">decisao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Os valores sao decisao do CEO. Nada vai para tela sem eles.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Definir quanto custa cada modulo em reais. So voce decide. Nenhum preco vai para tela sem isso.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menu com modulos travados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Itens nao comprados aparecem apagados com cadeado. Clique abre a mensagem de desejo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coracao do modelo comercial. Depende do catalogo e dos precos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Os modulos que a clinica nao comprou aparecem apagados com um cadeado, e clicar abre a oferta. E a vitrine da loja: voce ve o que nao comprou, e isso e o que faz querer comprar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mensagem de desejo com 48h e indicacao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descricao do beneficio, preco promocional valido 48h, valor cheio riscado, 10% por indicacao na adesao.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mensalidade nunca muda — desconto so na entrada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A mensagem que aparece ao clicar no cadeado: o que o modulo faz, o preco promocional valendo 48 horas, o valor cheio riscado e o desconto por indicacao.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login de licenciado (o segundo chapeu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segundo usuario do CEO, entrando na mesma clinica com a visao travada do cliente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dois logins, mesma clinica, lentes diferentes. Pagamento real de R$ 1 via Asaas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Um segundo usuario seu, entrando na mesma clinica, mas enxergando so o que um cliente enxergaria. Dois cracha, mesma porta, oculos diferentes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Painel do CEO com seletor de clinica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visao consolidada de todas as clinicas e troca de contexto para ver como o dono ve.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tenantContext ja modela isPlatformOwner + empresaId. Comecar somente-leitura nas outras clinicas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Painel onde voce ve todas as clinicas de uma vez e consegue entrar na visao de cada dona para ver o que ela ve.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Painel de bilhetagem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consumo por clinica, por periodo, por tipo. Atualizacao por LISTEN/NOTIFY do Postgres.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 dias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sem fornecedor novo. Com 12 clinicas o Postgres aguenta com folga.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Painel de quanto cada clinica consumiu, por periodo e por tipo, atualizando sozinho na tela.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upsell por limiar de uso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regra por modulo: metrica, limiar, mensagem, desconto. Dispara apos cada evento de consumo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oferece quando o uso prova que faz sentido. Observacao honesta, nao pressao.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quando o uso de um modulo passa de um limite, o sistema oferece o upgrade sozinho. Oferece quando o proprio uso ja provou que faz sentido, nao antes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zoho configurado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZOHO_ORG_ID e token de admin nas variaveis. Codigo de criacao de conta e alias ja existe.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precisa da conta Zoho e do token. Depois disso o sistema cria sozinho.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configurar a conta de e-mail corporativo. Depois disso o sistema cria os e-mails de cada clinica nova sozinho.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DNS automatico via Cloudflare API</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ao ativar uma clinica, o sistema cria os registros de DNS sem ninguem tocar no painel.</t>
+  </si>
+  <si>
     <t xml:space="preserve">3h</t>
   </si>
   <si>
-    <t xml:space="preserve">Os dois gravam scrypt$ hoje. Foi a armadilha que custou uma noite inteira.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Existem dois tipos de senha no sistema, guardados de jeitos diferentes, mas gravados com a MESMA etiqueta. E como dois frascos de remedio com o mesmo rotulo e conteudo diferente. Foi isso que fez seu login falhar por uma noite inteira. Isso poe rotulo diferente em cada frasco.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tela de login dentro do padaxor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tela propria chamando /api/collaborator/login e setCollabSession. O encanamento ja existe em collab-auth.ts.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entregue 30/07 no commit 3a38349, conferido: pages/login/index.tsx criado e CollaboratorGate passou a redirecionar.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tela de entrada propria do sistema, em vez da caixinha cinza do navegador. Ja entregue em 30/07.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Site vira botao, nao segundo login</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O login do site aponta para a tela do sistema em vez de autenticar por conta propria.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LIBERADO em 30/07: a tela do item 11 existe. Elimina o segundo formulario de autenticacao.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O botao Entrar do site deixa de pedir senha por conta propria e passa a levar a pessoa para a tela de entrada do sistema. Uma porta so em vez de duas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DNS do padaxor.com.br no Cloudflare</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trocar os servidores de nome no Registro.br pelos do Cloudflare.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15min</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Railway exige CNAME Flattening ou ALIAS para dominio raiz. Registro.br nao faz.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trocar quem cuida do endereco padaxor.com.br na internet. O registrador brasileiro nao faz um recurso que o servidor precisa; o Cloudflare faz, e e de graca.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dominio proprio apontando para o sistema</t>
-  </si>
-  <si>
-    <t xml:space="preserve">app.padaxor.com.br no Railway com certificado automatico.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AGUARDANDO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Depende do passo do Cloudflare.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fazer app.padaxor.com.br apontar para o sistema, com cadeado de seguranca automatico no navegador.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marca PAXTER para PADAXOR no painel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O painel do sistema ainda exibe PAXTER na identidade visual.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">parcial</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Titulo da aba e do aplicativo entregues 30/07 no commit 3a38349. As telas internas seguem no item 38.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O painel ainda mostrava o nome antigo PAXTER. Titulo da aba corrigido em 30/07; o resto das telas segue no item 38.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Porta da area do paciente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O site nao tem entrada para /api/area-paciente, que tem 12 rotas prontas no servidor.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quarta porta do produto inteira sem macaneta.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O servidor ja tem doze portas prontas para a area do paciente, mas o site nao tem nenhum botao que leve ate elas. E uma porta inteira construida e sem macaneta.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Indice unico em lower(login_username)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Impede dois colaboradores com o mesmo usuario. Erro 23505 traduzido em 409.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prevencao. Nao foi a causa do bug de hoje — nao havia duplicata.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Impedir que dois colaboradores tenham o mesmo nome de usuario. Prevencao: nao foi a causa do problema de hoje, mas seria a causa do de amanha.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ligar o registro de consumo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comecar a gravar em consumo_eventos, que ja existe com empresa_id, custo e idempotencia.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P2 medio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sem historico nao ha painel. Historico nao se cria retroativamente. Espera o RLS do Dr. Code.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comecar a anotar quanto cada clinica usa do sistema. Sem anotar desde ja, nao existe historico depois: historico nao se cria para tras.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Catalogo de modulos com precos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tabela de modulos: nome, beneficio, valor de adesao, valor promocional, mensalidade.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">decisao</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Os valores sao decisao do CEO. Nada vai para tela sem eles.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Definir quanto custa cada modulo em reais. So voce decide. Nenhum preco vai para tela sem isso.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Menu com modulos travados</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Itens nao comprados aparecem apagados com cadeado. Clique abre a mensagem de desejo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coracao do modelo comercial. Depende do catalogo e dos precos.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Os modulos que a clinica nao comprou aparecem apagados com um cadeado, e clicar abre a oferta. E a vitrine da loja: voce ve o que nao comprou, e isso e o que faz querer comprar.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mensagem de desejo com 48h e indicacao</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Descricao do beneficio, preco promocional valido 48h, valor cheio riscado, 10% por indicacao na adesao.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mensalidade nunca muda — desconto so na entrada.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A mensagem que aparece ao clicar no cadeado: o que o modulo faz, o preco promocional valendo 48 horas, o valor cheio riscado e o desconto por indicacao.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Login de licenciado (o segundo chapeu)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Segundo usuario do CEO, entrando na mesma clinica com a visao travada do cliente.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dois logins, mesma clinica, lentes diferentes. Pagamento real de R$ 1 via Asaas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Um segundo usuario seu, entrando na mesma clinica, mas enxergando so o que um cliente enxergaria. Dois cracha, mesma porta, oculos diferentes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Painel do CEO com seletor de clinica</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Visao consolidada de todas as clinicas e troca de contexto para ver como o dono ve.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tenantContext ja modela isPlatformOwner + empresaId. Comecar somente-leitura nas outras clinicas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Painel onde voce ve todas as clinicas de uma vez e consegue entrar na visao de cada dona para ver o que ela ve.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Painel de bilhetagem</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Consumo por clinica, por periodo, por tipo. Atualizacao por LISTEN/NOTIFY do Postgres.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 dias</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sem fornecedor novo. Com 12 clinicas o Postgres aguenta com folga.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Painel de quanto cada clinica consumiu, por periodo e por tipo, atualizando sozinho na tela.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Upsell por limiar de uso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Regra por modulo: metrica, limiar, mensagem, desconto. Dispara apos cada evento de consumo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oferece quando o uso prova que faz sentido. Observacao honesta, nao pressao.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quando o uso de um modulo passa de um limite, o sistema oferece o upgrade sozinho. Oferece quando o proprio uso ja provou que faz sentido, nao antes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zoho configurado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZOHO_ORG_ID e token de admin nas variaveis. Codigo de criacao de conta e alias ja existe.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">30min</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Precisa da conta Zoho e do token. Depois disso o sistema cria sozinho.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Configurar a conta de e-mail corporativo. Depois disso o sistema cria os e-mails de cada clinica nova sozinho.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DNS automatico via Cloudflare API</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ao ativar uma clinica, o sistema cria os registros de DNS sem ninguem tocar no painel.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Depende do Cloudflare ser o provedor de DNS.</t>
   </si>
   <si>
@@ -1333,6 +1336,18 @@
   </si>
   <si>
     <t xml:space="preserve">Dr. Chat (ChatGPT) entrou no quadro por decisao do CEO. Territorio escolhido para NAO sobrepor ninguem: peca avulsa e auditoria independente, entregue na doca, sem commitar. Modelo de familia diferente lendo a mesma spec pega o que o autor nao viu.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONCLUIDO (fase 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Causa raiz PROVADA por teste, nao por leitura: os dois esquemas gravavam scrypt$ e derivavam de formas incompativeis, um entregando o salt como string e o outro como buffer. O teste 1 do commit df4c998 demonstra chaves diferentes para mesmo salt e mesma senha. Corrigido sem regravar nenhuma senha: mudou o rotulo, nao a derivacao.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">commit df4c998</t>
   </si>
   <si>
     <t xml:space="preserve">42-48</t>
@@ -2877,34 +2892,34 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="n">
+      <c r="A14" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F14" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="G14" s="5" t="s">
+      <c r="F14" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G14" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="H14" s="5" t="s">
+      <c r="H14" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="I14" s="5" t="s">
+      <c r="I14" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="J14" s="5" t="s">
+      <c r="J14" s="4" t="s">
         <v>67</v>
       </c>
     </row>
@@ -3443,13 +3458,13 @@
         <v>107</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>65</v>
+        <v>151</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J31" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3457,16 +3472,16 @@
         <v>28</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D32" s="6" t="s">
         <v>14</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>87</v>
@@ -3475,13 +3490,13 @@
         <v>107</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I32" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J32" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3489,10 +3504,10 @@
         <v>29</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D33" s="6" t="s">
         <v>28</v>
@@ -3510,10 +3525,10 @@
         <v>54</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J33" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3521,13 +3536,13 @@
         <v>30</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E34" s="5" t="s">
         <v>15</v>
@@ -3536,16 +3551,16 @@
         <v>53</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H34" s="5" t="s">
         <v>97</v>
       </c>
       <c r="I34" s="5" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J34" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3553,31 +3568,31 @@
         <v>31</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>43</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F35" s="5" t="s">
         <v>53</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H35" s="5" t="s">
         <v>97</v>
       </c>
       <c r="I35" s="5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J35" s="5" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3585,10 +3600,10 @@
         <v>32</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>28</v>
@@ -3600,16 +3615,16 @@
         <v>53</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="I36" s="5" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J36" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3617,31 +3632,31 @@
         <v>33</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>28</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F37" s="6" t="s">
         <v>87</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H37" s="6" t="s">
         <v>60</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J37" s="6" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3649,10 +3664,10 @@
         <v>34</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>23</v>
@@ -3664,16 +3679,16 @@
         <v>53</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H38" s="5" t="s">
         <v>112</v>
       </c>
       <c r="I38" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="J38" s="5" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3681,10 +3696,10 @@
         <v>35</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>28</v>
@@ -3696,16 +3711,16 @@
         <v>53</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H39" s="5" t="s">
         <v>60</v>
       </c>
       <c r="I39" s="5" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J39" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3713,13 +3728,13 @@
         <v>36</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E40" s="4" t="s">
         <v>15</v>
@@ -3728,16 +3743,16 @@
         <v>16</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H40" s="4" t="s">
         <v>15</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3745,10 +3760,10 @@
         <v>37</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>14</v>
@@ -3766,10 +3781,10 @@
         <v>60</v>
       </c>
       <c r="I41" s="5" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J41" s="5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3777,10 +3792,10 @@
         <v>40</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>14</v>
@@ -3798,10 +3813,10 @@
         <v>18</v>
       </c>
       <c r="I42" s="4" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="J42" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3809,10 +3824,10 @@
         <v>42</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>14</v>
@@ -3827,13 +3842,13 @@
         <v>17</v>
       </c>
       <c r="H43" s="5" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I43" s="5" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="J43" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3841,10 +3856,10 @@
         <v>43</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>14</v>
@@ -3859,13 +3874,13 @@
         <v>44</v>
       </c>
       <c r="H44" s="5" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I44" s="5" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J44" s="5" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3873,16 +3888,16 @@
         <v>44</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D45" s="6" t="s">
         <v>28</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F45" s="6" t="s">
         <v>87</v>
@@ -3891,13 +3906,13 @@
         <v>44</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I45" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J45" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3905,16 +3920,16 @@
         <v>45</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D46" s="6" t="s">
         <v>14</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>87</v>
@@ -3923,13 +3938,13 @@
         <v>107</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I46" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="J46" s="6" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3937,16 +3952,16 @@
         <v>46</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D47" s="6" t="s">
         <v>14</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F47" s="6" t="s">
         <v>87</v>
@@ -3955,13 +3970,13 @@
         <v>107</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I47" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J47" s="6" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3969,10 +3984,10 @@
         <v>47</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D48" s="5" t="s">
         <v>14</v>
@@ -3987,13 +4002,13 @@
         <v>44</v>
       </c>
       <c r="H48" s="5" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I48" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="J48" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4001,10 +4016,10 @@
         <v>48</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>28</v>
@@ -4022,10 +4037,10 @@
         <v>54</v>
       </c>
       <c r="I49" s="5" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J49" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4033,10 +4048,10 @@
         <v>41</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>14</v>
@@ -4054,10 +4069,10 @@
         <v>60</v>
       </c>
       <c r="I50" s="5" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J50" s="5" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4065,10 +4080,10 @@
         <v>39</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D51" s="5" t="s">
         <v>28</v>
@@ -4083,13 +4098,13 @@
         <v>107</v>
       </c>
       <c r="H51" s="5" t="s">
-        <v>65</v>
+        <v>151</v>
       </c>
       <c r="I51" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J51" s="5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4097,10 +4112,10 @@
         <v>38</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D52" s="5" t="s">
         <v>14</v>
@@ -4115,41 +4130,41 @@
         <v>44</v>
       </c>
       <c r="H52" s="5" t="s">
-        <v>65</v>
+        <v>151</v>
       </c>
       <c r="I52" s="5" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="J52" s="5" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="7" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="8" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C55" s="9" t="n">
         <f aca="false">COUNTIF(F5:F52,"CONCLUIDO")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="8" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C56" s="9" t="n">
         <f aca="false">COUNTIF(F5:F52,"A FAZER")</f>
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="8" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C57" s="9" t="n">
         <f aca="false">COUNTIF(F5:F52,"AGUARDANDO")</f>
@@ -4158,7 +4173,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="8" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C58" s="9" t="n">
         <f aca="false">COUNTA(A5:A52)</f>
@@ -4208,7 +4223,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4217,7 +4232,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4226,19 +4241,19 @@
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4246,16 +4261,16 @@
         <v>23</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4263,33 +4278,33 @@
         <v>28</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4297,111 +4312,111 @@
         <v>43</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>287</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>288</v>
+      </c>
+      <c r="E12" s="10" t="s">
         <v>289</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>206</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>286</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>287</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
@@ -4410,7 +4425,7 @@
     </row>
     <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B18" s="11"/>
       <c r="C18" s="11"/>
@@ -4419,7 +4434,7 @@
     </row>
     <row r="19" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B19" s="11"/>
       <c r="C19" s="11"/>
@@ -4428,7 +4443,7 @@
     </row>
     <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B20" s="11"/>
       <c r="C20" s="11"/>
@@ -4437,7 +4452,7 @@
     </row>
     <row r="21" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B21" s="11"/>
       <c r="C21" s="11"/>
@@ -4481,7 +4496,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4490,7 +4505,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4502,16 +4517,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4519,13 +4534,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E5" s="12"/>
     </row>
@@ -4534,13 +4549,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E6" s="12"/>
     </row>
@@ -4549,10 +4564,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>122</v>
@@ -4564,10 +4579,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>122</v>
@@ -4579,13 +4594,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E9" s="12"/>
     </row>
@@ -4594,13 +4609,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E10" s="12"/>
     </row>
@@ -4609,13 +4624,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E11" s="12"/>
     </row>
@@ -4624,13 +4639,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E12" s="12"/>
     </row>
@@ -4639,13 +4654,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E13" s="12"/>
     </row>
@@ -4654,36 +4669,36 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E14" s="12"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="13" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>15</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
   </sheetData>
@@ -4715,78 +4730,78 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
   </sheetData>
@@ -4819,7 +4834,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4827,7 +4842,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4835,128 +4850,128 @@
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
   </sheetData>
@@ -4979,7 +4994,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -4993,7 +5008,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5005,7 +5020,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -5017,33 +5032,33 @@
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>28</v>
@@ -5052,30 +5067,30 @@
         <v>15</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>15</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>28</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>7</v>
@@ -5087,15 +5102,15 @@
         <v>53</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>28</v>
@@ -5113,21 +5128,21 @@
         <v>87</v>
       </c>
       <c r="G7" s="10" t="s">
+        <v>407</v>
+      </c>
+      <c r="H7" s="10" t="s">
         <v>406</v>
-      </c>
-      <c r="H7" s="10" t="s">
-        <v>405</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>28</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>7</v>
@@ -5139,15 +5154,15 @@
         <v>87</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>14</v>
@@ -5165,21 +5180,21 @@
         <v>16</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>7</v>
@@ -5191,21 +5206,21 @@
         <v>16</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>28</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="D11" s="10" t="s">
         <v>7</v>
@@ -5217,24 +5232,24 @@
         <v>53</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>28</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>15</v>
@@ -5243,24 +5258,24 @@
         <v>53</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>28</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>15</v>
@@ -5269,21 +5284,21 @@
         <v>53</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>28</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>5</v>
@@ -5292,24 +5307,24 @@
         <v>28</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>28</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D15" s="10" t="s">
         <v>7</v>
@@ -5321,15 +5336,15 @@
         <v>16</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>28</v>
@@ -5338,24 +5353,24 @@
         <v>15</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>28</v>
@@ -5364,111 +5379,111 @@
         <v>15</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>28</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>399</v>
+        <v>7</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>15</v>
+        <v>53</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>53</v>
+        <v>436</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>7</v>
+        <v>400</v>
       </c>
       <c r="E19" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F19" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="F19" s="10" t="s">
-        <v>16</v>
-      </c>
       <c r="G19" s="10" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>399</v>
+        <v>7</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>15</v>
+        <v>53</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>53</v>
+        <v>16</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>28</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>437</v>
+        <v>445</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>15</v>
@@ -5477,93 +5492,93 @@
         <v>53</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="H21" s="10" t="s">
-        <v>422</v>
+        <v>447</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>28</v>
       </c>
       <c r="C22" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="E22" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D22" s="5" t="s">
-        <v>444</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>445</v>
-      </c>
       <c r="F22" s="5" t="s">
-        <v>446</v>
+        <v>53</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>448</v>
+        <v>423</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B23" s="10" t="s">
         <v>28</v>
       </c>
       <c r="C23" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D23" s="10" t="s">
         <v>449</v>
       </c>
-      <c r="D23" s="10" t="s">
-        <v>399</v>
-      </c>
       <c r="E23" s="10" t="s">
-        <v>15</v>
+        <v>450</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>53</v>
+        <v>451</v>
       </c>
       <c r="G23" s="10" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="H23" s="10" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>28</v>
       </c>
       <c r="C24" s="5" t="s">
+        <v>454</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="E24" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D24" s="5" t="s">
-        <v>430</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>432</v>
-      </c>
       <c r="F24" s="5" t="s">
-        <v>452</v>
+        <v>53</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>422</v>
+        <v>456</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B25" s="10" t="s">
         <v>28</v>
@@ -5572,35 +5587,61 @@
         <v>15</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>454</v>
+        <v>431</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>455</v>
+        <v>433</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="G25" s="10" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="H25" s="10" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="16" t="s">
-        <v>458</v>
-      </c>
-      <c r="B26" s="17"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
-      <c r="G26" s="17"/>
-      <c r="H26" s="17"/>
+        <v>423</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="5" t="s">
+        <v>410</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>460</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>461</v>
+      </c>
+      <c r="G26" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="16" t="s">
+        <v>463</v>
+      </c>
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="17"/>
+      <c r="H27" s="17"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H25"/>
+  <autoFilter ref="A4:H26"/>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
@@ -5633,7 +5674,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>459</v>
+        <v>464</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5642,7 +5683,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>460</v>
+        <v>465</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -5651,602 +5692,602 @@
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>461</v>
+        <v>466</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>462</v>
+        <v>467</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>463</v>
+        <v>468</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>464</v>
+        <v>469</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>465</v>
+        <v>470</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>466</v>
+        <v>471</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>467</v>
+        <v>472</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>470</v>
+        <v>475</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>471</v>
+        <v>476</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>472</v>
+        <v>477</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>473</v>
+        <v>478</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>476</v>
+        <v>481</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>477</v>
+        <v>482</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>478</v>
+        <v>483</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>479</v>
+        <v>484</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>480</v>
+        <v>485</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>481</v>
+        <v>486</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>482</v>
+        <v>487</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>483</v>
+        <v>488</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>484</v>
+        <v>489</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>486</v>
+        <v>491</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>487</v>
+        <v>492</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>488</v>
+        <v>493</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>489</v>
+        <v>494</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>491</v>
+        <v>496</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>492</v>
+        <v>497</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>493</v>
+        <v>498</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>494</v>
+        <v>499</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>496</v>
+        <v>501</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>497</v>
+        <v>502</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>498</v>
+        <v>503</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>499</v>
+        <v>504</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>500</v>
+        <v>505</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>501</v>
+        <v>506</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>503</v>
+        <v>508</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>505</v>
+        <v>510</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>506</v>
+        <v>511</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>507</v>
+        <v>512</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>508</v>
+        <v>513</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>509</v>
+        <v>514</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>510</v>
+        <v>515</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>512</v>
+        <v>517</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>513</v>
+        <v>518</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>514</v>
+        <v>519</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>515</v>
+        <v>520</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>516</v>
+        <v>521</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>517</v>
+        <v>522</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>518</v>
+        <v>523</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>519</v>
+        <v>524</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>520</v>
+        <v>525</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>521</v>
+        <v>526</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>522</v>
+        <v>527</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>523</v>
+        <v>528</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>524</v>
+        <v>529</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>525</v>
+        <v>530</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>526</v>
+        <v>531</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>527</v>
+        <v>532</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>528</v>
+        <v>533</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>529</v>
+        <v>534</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>530</v>
+        <v>535</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>531</v>
+        <v>536</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>532</v>
+        <v>537</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>533</v>
+        <v>538</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>534</v>
+        <v>539</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>535</v>
+        <v>540</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>536</v>
+        <v>541</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>537</v>
+        <v>542</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>538</v>
+        <v>543</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>539</v>
+        <v>544</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>540</v>
+        <v>545</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>541</v>
+        <v>546</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>542</v>
+        <v>547</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>543</v>
+        <v>548</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>545</v>
+        <v>550</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>546</v>
+        <v>551</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>547</v>
+        <v>552</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>548</v>
+        <v>553</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>549</v>
+        <v>554</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>550</v>
+        <v>555</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>551</v>
+        <v>556</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>552</v>
+        <v>557</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>553</v>
+        <v>558</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>554</v>
+        <v>559</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>555</v>
+        <v>560</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>556</v>
+        <v>561</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>557</v>
+        <v>562</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>558</v>
+        <v>563</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>559</v>
+        <v>564</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>560</v>
+        <v>565</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>561</v>
+        <v>566</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>562</v>
+        <v>567</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>563</v>
+        <v>568</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>564</v>
+        <v>569</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>566</v>
+        <v>571</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>567</v>
+        <v>572</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>568</v>
+        <v>573</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>570</v>
+        <v>575</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>571</v>
+        <v>576</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>573</v>
+        <v>578</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>575</v>
+        <v>580</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>576</v>
+        <v>581</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>577</v>
+        <v>582</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>578</v>
+        <v>583</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>579</v>
+        <v>584</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>580</v>
+        <v>585</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>581</v>
+        <v>586</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>582</v>
+        <v>587</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>583</v>
+        <v>588</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>584</v>
+        <v>589</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>585</v>
+        <v>590</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>586</v>
+        <v>591</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>587</v>
+        <v>592</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>588</v>
+        <v>593</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>589</v>
+        <v>594</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>590</v>
+        <v>595</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>591</v>
+        <v>596</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>592</v>
+        <v>597</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>593</v>
+        <v>598</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>594</v>
+        <v>599</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>595</v>
+        <v>600</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>596</v>
+        <v>601</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>598</v>
+        <v>603</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>599</v>
+        <v>604</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>600</v>
+        <v>605</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>601</v>
+        <v>606</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>602</v>
+        <v>607</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>603</v>
+        <v>608</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>604</v>
+        <v>609</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>605</v>
+        <v>610</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>606</v>
+        <v>611</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>607</v>
+        <v>612</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>608</v>
+        <v>613</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>609</v>
+        <v>614</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>610</v>
+        <v>615</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>611</v>
+        <v>616</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>612</v>
+        <v>617</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>613</v>
+        <v>618</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>614</v>
+        <v>619</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>615</v>
+        <v>620</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>616</v>
+        <v>621</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>617</v>
+        <v>622</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>618</v>
+        <v>623</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>619</v>
+        <v>624</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>620</v>
+        <v>625</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>621</v>
+        <v>626</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>622</v>
+        <v>627</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>623</v>
+        <v>628</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>624</v>
+        <v>629</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>625</v>
+        <v>630</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>626</v>
+        <v>631</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>627</v>
+        <v>632</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>628</v>
+        <v>633</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>629</v>
+        <v>634</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>630</v>
+        <v>635</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>631</v>
+        <v>636</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>632</v>
+        <v>637</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>633</v>
+        <v>638</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>634</v>
+        <v>639</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="16" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="B39" s="17"/>
       <c r="C39" s="17"/>

</xml_diff>